<commit_message>
docs(clinic): leave the annual half-body package unwired, by decision
The two 12-session half-body packages were given names that say the same thing,
and one phrase was given to both — which an import refuses, because a name that
reaches two rows is how a patient is booked into the treatment they did not ask
for. The client has settled it by dropping one side: DT020 carries no Arabic
name at all.

Its row stays in the list, empty, so the decision reads as a decision rather
than as something nobody got to. It still answers to its English catalogue name,
so it remains bookable; it just cannot be reached by an Arabic phrase.

The effect on the other side is clean: every Arabic half-body phrasing now
reaches DT023 outright with no clarifying question. Over the demo's 23 phrases,
22 resolve, one asks (a bare ليزر against nine packages), and none reach
nothing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011RAsvFWVPoUvpmeCiYqu8T
</commit_message>
<xml_diff>
--- a/docs/DermaClub_Aliases_DRAFT_2026-08-28.xlsx
+++ b/docs/DermaClub_Aliases_DRAFT_2026-08-28.xlsx
@@ -1329,19 +1329,15 @@
           <t>Annual Half Body (12 Sessions)</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>ليزر سنوي 12 جلسة هاف بودي|ليزر نص الجسم 12 جلسة سنوي</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>client-approved</t>
+          <t>not-wired</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Q1, answered. The clinic gave ليزر 12 جلسة نص الجسم to this package and to DT023; one string cannot name two rows, so it sits here in the clinic's own longer form and on DT023 in theirs. A patient using the shorter phrase reaches both and is asked which.</t>
+          <t>Deliberately left unwired at the clinic's instruction. The row stays in the list so the decision is visible rather than looking like an omission: DT020 answers to its English catalogue name and to nothing in Arabic, and every Arabic half-body phrase now reaches DT023 alone.</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1410,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Q1, answered. See DT020 for the one phrase the clinic gave to both.</t>
+          <t>Q1, answered. The only half-body package with Arabic names: DT020 is deliberately unwired, so every Arabic phrasing lands here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(clinic): the Biostimulator gets the clinic's own word
محفزات الكولاجين, answered on the review page, with the singular محفز الكولاجين
beside it because patients write either and the matcher reads them as different
words. The transliterations stay behind both — they are also what people type.

That closes the last open question on the alias list. Over the demo's phrases,
now 24 of them: 23 resolve, one asks (a bare ليزر against nine packages), none
reach nothing. Nothing is imported and the client's workbook is still untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011RAsvFWVPoUvpmeCiYqu8T
</commit_message>
<xml_diff>
--- a/docs/DermaClub_Aliases_DRAFT_2026-08-28.xlsx
+++ b/docs/DermaClub_Aliases_DRAFT_2026-08-28.xlsx
@@ -1166,17 +1166,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>بيوستيميوليتور|بيو ستيميوليتور</t>
+          <t>محفزات الكولاجين|محفز الكولاجين|بيوستيميوليتور|بيو ستيميوليتور</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>drafted</t>
+          <t>client-approved</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Transliteration only. Many patients call this محفزات الكولاجين — needs the clinic's word before it goes in (open question 3).</t>
+          <t>Q3, answered by the clinic. Their words first, the transliterations kept behind them: patients type both.</t>
         </is>
       </c>
     </row>

</xml_diff>